<commit_message>
update data and workflow
</commit_message>
<xml_diff>
--- a/OrangeHRM/Data/OrangeHRM_Login.xlsx
+++ b/OrangeHRM/Data/OrangeHRM_Login.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29922"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Life\Learning\Esprit\PFE\Project\TessanTIS\TessanTIS.OrangeHRM.Data.Impl\Data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Life\Learning\Esprit\PFE\Project\TessanTIS\OrangeHRM\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0E92A803-B951-415C-B64F-A73585DBE19E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4CBC6BA9-5198-48A6-A0E4-85235C2EC9B8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-6540" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{56F28EB9-5BA8-428B-AB16-A5C338242BCA}"/>
+    <workbookView xWindow="28680" yWindow="-6540" windowWidth="29040" windowHeight="15720" xr2:uid="{56F28EB9-5BA8-428B-AB16-A5C338242BCA}"/>
   </bookViews>
   <sheets>
     <sheet name="OrangeHRM_Login_TC001" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="40">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="42">
   <si>
     <t>Steps</t>
   </si>
@@ -157,6 +157,12 @@
   </si>
   <si>
     <t>There are 8 errors</t>
+  </si>
+  <si>
+    <t>Admin</t>
+  </si>
+  <si>
+    <t>admin123</t>
   </si>
 </sst>
 </file>
@@ -590,10 +596,10 @@
         <v>16</v>
       </c>
       <c r="B2" t="s">
-        <v>17</v>
+        <v>40</v>
       </c>
       <c r="C2" t="s">
-        <v>17</v>
+        <v>41</v>
       </c>
     </row>
     <row r="3" spans="1:16" x14ac:dyDescent="0.35">
@@ -825,12 +831,9 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1037,15 +1040,19 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A4EF81E7-E39B-43E7-BD54-614E952B9C15}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5E949F8F-1265-4F7D-8B3B-442451397EE3}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -1070,10 +1077,9 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5E949F8F-1265-4F7D-8B3B-442451397EE3}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A4EF81E7-E39B-43E7-BD54-614E952B9C15}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>